<commit_message>
À partir du tuto 12, on se  passe de loader basic pour pouvoir utiliser plus de mémoire
</commit_message>
<xml_diff>
--- a/docs/CPC Z80 Tools.xlsx
+++ b/docs/CPC Z80 Tools.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <workbookPr/>
   <bookViews>
-    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="1"/>
+    <workbookView xWindow="360" yWindow="15" windowWidth="20955" windowHeight="9720" activeTab="0"/>
   </bookViews>
   <sheets>
     <sheet name="RAM CPC 6128" sheetId="1" state="visible" r:id="rId1"/>
@@ -131,7 +131,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="18">
+  <cellXfs count="14">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -146,22 +146,14 @@
     <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="164" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
       <protection hidden="0" locked="1"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="165" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-      <protection hidden="0" locked="1"/>
-    </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0">
       <protection hidden="0" locked="1"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
       <protection hidden="0" locked="1"/>
@@ -178,9 +170,6 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
       <protection hidden="0" locked="1"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -701,7 +690,7 @@
         <v>0</v>
       </c>
       <c r="B2" s="5" t="str">
-        <f>DEC2HEX(A2)</f>
+        <f t="shared" ref="B2:B9" si="0">DEC2HEX(A2)</f>
         <v>0</v>
       </c>
       <c r="C2" t="s">
@@ -709,45 +698,45 @@
       </c>
     </row>
     <row r="3" ht="14.25">
-      <c r="A3" s="6">
+      <c r="A3" s="4">
         <v>63</v>
       </c>
-      <c r="B3" s="7" t="str">
-        <f>DEC2HEX(A3)</f>
+      <c r="B3" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>3F</v>
       </c>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="6">
+      <c r="A4" s="4">
         <v>64</v>
       </c>
-      <c r="B4" s="7" t="str">
-        <f>DEC2HEX(A4)</f>
+      <c r="B4" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>40</v>
       </c>
       <c r="C4" t="s">
         <v>4</v>
       </c>
-      <c r="D4" s="8"/>
+      <c r="D4" s="7"/>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="6">
+      <c r="A5" s="4">
         <f>HEX2DEC("16f")</f>
         <v>367</v>
       </c>
-      <c r="B5" s="7" t="str">
-        <f>DEC2HEX(A5)</f>
+      <c r="B5" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>16F</v>
       </c>
-      <c r="D5" s="8"/>
+      <c r="D5" s="7"/>
     </row>
     <row r="6" ht="14.25">
       <c r="A6" s="4">
         <f>HEX2DEC(170)</f>
         <v>368</v>
       </c>
-      <c r="B6" s="9" t="str">
-        <f>DEC2HEX(A6)</f>
+      <c r="B6" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>170</v>
       </c>
       <c r="C6" t="s">
@@ -763,8 +752,8 @@
         <f>A9-1</f>
         <v>8191</v>
       </c>
-      <c r="B8" s="9" t="str">
-        <f>DEC2HEX(A8)</f>
+      <c r="B8" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>1FFF</v>
       </c>
       <c r="C8" t="s">
@@ -775,12 +764,12 @@
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="6">
+      <c r="A9" s="4">
         <f>HEX2DEC("2000")</f>
         <v>8192</v>
       </c>
-      <c r="B9" s="7" t="str">
-        <f>DEC2HEX(A9)</f>
+      <c r="B9" s="6" t="str">
+        <f t="shared" si="0"/>
         <v>2000</v>
       </c>
       <c r="C9" t="s">
@@ -792,26 +781,26 @@
     </row>
     <row r="10" ht="14.25">
       <c r="A10" s="4"/>
-      <c r="B10" s="9"/>
-      <c r="H10" s="10">
+      <c r="B10" s="6"/>
+      <c r="H10" s="8">
         <v>16348</v>
       </c>
     </row>
     <row r="11" ht="14.25">
       <c r="A11" s="4"/>
-      <c r="B11" s="9"/>
+      <c r="B11" s="6"/>
       <c r="H11">
         <f>H8-H9-H10</f>
         <v>1731</v>
       </c>
     </row>
     <row r="12" ht="14.25">
-      <c r="A12" s="6">
-        <f>A13-16384</f>
+      <c r="A12" s="4">
+        <f t="shared" ref="A12:A13" si="1">A13-16384</f>
         <v>9851</v>
       </c>
-      <c r="B12" s="7" t="str">
-        <f>DEC2HEX(A12)</f>
+      <c r="B12" s="6" t="str">
+        <f t="shared" ref="B12:B21" si="2">DEC2HEX(A12)</f>
         <v>267B</v>
       </c>
       <c r="C12" t="s">
@@ -820,14 +809,14 @@
     </row>
     <row r="13" ht="14.25">
       <c r="A13" s="4">
-        <f>A14-16384</f>
+        <f t="shared" si="1"/>
         <v>26235</v>
       </c>
-      <c r="B13" s="9" t="str">
-        <f>DEC2HEX(A13)</f>
+      <c r="B13" s="6" t="str">
+        <f t="shared" si="2"/>
         <v>667B</v>
       </c>
-      <c r="C13" s="11" t="s">
+      <c r="C13" s="7" t="s">
         <v>9</v>
       </c>
     </row>
@@ -835,8 +824,8 @@
       <c r="A14" s="4">
         <v>42619</v>
       </c>
-      <c r="B14" s="9" t="str">
-        <f>DEC2HEX(A14)</f>
+      <c r="B14" s="6" t="str">
+        <f t="shared" si="2"/>
         <v>A67B</v>
       </c>
       <c r="C14" t="s">
@@ -852,8 +841,8 @@
         <f>HEX2DEC("a660")</f>
         <v>42592</v>
       </c>
-      <c r="B16" s="9" t="str">
-        <f>DEC2HEX(A16)</f>
+      <c r="B16" s="6" t="str">
+        <f t="shared" si="2"/>
         <v>A660</v>
       </c>
       <c r="C16" t="s">
@@ -877,12 +866,12 @@
       <c r="B20" s="5"/>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="12">
+      <c r="A21" s="9">
         <f>HEX2DEC("c000")</f>
         <v>49152</v>
       </c>
-      <c r="B21" s="9" t="str">
-        <f>DEC2HEX(A21)</f>
+      <c r="B21" s="6" t="str">
+        <f t="shared" si="2"/>
         <v>C000</v>
       </c>
       <c r="C21" t="s">
@@ -955,7 +944,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac">
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.25"/>
   <cols>
     <col customWidth="1" min="14" max="14" width="51.140625"/>
   </cols>
@@ -993,265 +982,265 @@
         <v>13</v>
       </c>
     </row>
-    <row r="4" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A4" s="13"/>
-      <c r="B4" s="14">
-        <v>0</v>
-      </c>
-      <c r="C4" s="14">
-        <v>0</v>
-      </c>
-      <c r="D4" s="14">
-        <v>0</v>
-      </c>
-      <c r="E4" s="14">
-        <v>1</v>
-      </c>
-      <c r="F4" s="14">
-        <v>1</v>
-      </c>
-      <c r="G4" s="14">
-        <v>0</v>
-      </c>
-      <c r="H4" s="14">
-        <v>0</v>
-      </c>
-      <c r="I4" s="14">
-        <v>0</v>
-      </c>
-      <c r="J4" s="13"/>
-      <c r="K4" s="13">
-        <f>(B4*128+C4*64+D4*32+E4*16+F4*8+G4*4+H4*2+I4*1)</f>
-        <v>24</v>
-      </c>
-      <c r="L4" s="13"/>
-      <c r="M4" s="13"/>
-      <c r="N4" s="15" t="str">
+    <row r="4" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A4" s="10"/>
+      <c r="B4" s="11">
+        <v>1</v>
+      </c>
+      <c r="C4" s="11">
+        <v>1</v>
+      </c>
+      <c r="D4" s="11">
+        <v>1</v>
+      </c>
+      <c r="E4" s="11">
+        <v>1</v>
+      </c>
+      <c r="F4" s="11">
+        <v>1</v>
+      </c>
+      <c r="G4" s="11">
+        <v>1</v>
+      </c>
+      <c r="H4" s="11">
+        <v>1</v>
+      </c>
+      <c r="I4" s="11">
+        <v>1</v>
+      </c>
+      <c r="J4" s="10"/>
+      <c r="K4" s="10">
+        <f t="shared" ref="K4:K9" si="3">(B4*128+C4*64+D4*32+E4*16+F4*8+G4*4+H4*2+I4*1)</f>
+        <v>255</v>
+      </c>
+      <c r="L4" s="10"/>
+      <c r="M4" s="10"/>
+      <c r="N4" s="12" t="str">
         <f>"DB "&amp;K4&amp;","&amp;K5&amp;","&amp;K6&amp;","&amp;K7&amp;","&amp;K8&amp;","&amp;K9&amp;","&amp;K10&amp;","&amp;K11</f>
-        <v xml:space="preserve">DB 24,60,126,255,153,153,159,255</v>
-      </c>
-      <c r="O4" s="13"/>
-      <c r="P4" s="13"/>
-    </row>
-    <row r="5" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A5" s="13"/>
-      <c r="B5" s="16">
-        <v>0</v>
-      </c>
-      <c r="C5" s="16">
-        <v>0</v>
-      </c>
-      <c r="D5" s="16">
-        <v>1</v>
-      </c>
-      <c r="E5" s="16">
-        <v>1</v>
-      </c>
-      <c r="F5" s="16">
-        <v>1</v>
-      </c>
-      <c r="G5" s="16">
-        <v>1</v>
-      </c>
-      <c r="H5" s="16">
-        <v>0</v>
-      </c>
-      <c r="I5" s="16">
-        <v>0</v>
-      </c>
-      <c r="J5" s="13"/>
-      <c r="K5" s="13">
-        <f>(B5*128+C5*64+D5*32+E5*16+F5*8+G5*4+H5*2+I5*1)</f>
-        <v>60</v>
-      </c>
-      <c r="L5" s="13"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="13"/>
-      <c r="O5" s="13"/>
-      <c r="P5" s="13"/>
-    </row>
-    <row r="6" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A6" s="13"/>
-      <c r="B6" s="16">
-        <v>0</v>
-      </c>
-      <c r="C6" s="16">
-        <v>1</v>
-      </c>
-      <c r="D6" s="16">
-        <v>1</v>
-      </c>
-      <c r="E6" s="16">
-        <v>1</v>
-      </c>
-      <c r="F6" s="16">
-        <v>1</v>
-      </c>
-      <c r="G6" s="16">
-        <v>1</v>
-      </c>
-      <c r="H6" s="16">
-        <v>1</v>
-      </c>
-      <c r="I6" s="16">
-        <v>0</v>
-      </c>
-      <c r="K6" s="13">
-        <f>(B6*128+C6*64+D6*32+E6*16+F6*8+G6*4+H6*2+I6*1)</f>
-        <v>126</v>
-      </c>
-    </row>
-    <row r="7" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A7" s="13"/>
-      <c r="B7" s="16">
-        <v>1</v>
-      </c>
-      <c r="C7" s="16">
-        <v>1</v>
-      </c>
-      <c r="D7" s="16">
-        <v>1</v>
-      </c>
-      <c r="E7" s="16">
-        <v>1</v>
-      </c>
-      <c r="F7" s="16">
-        <v>1</v>
-      </c>
-      <c r="G7" s="16">
-        <v>1</v>
-      </c>
-      <c r="H7" s="16">
-        <v>1</v>
-      </c>
-      <c r="I7" s="16">
-        <v>1</v>
-      </c>
-      <c r="K7" s="13">
-        <f>(B7*128+C7*64+D7*32+E7*16+F7*8+G7*4+H7*2+I7*1)</f>
-        <v>255</v>
-      </c>
-    </row>
-    <row r="8" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A8" s="13"/>
-      <c r="B8" s="16">
-        <v>1</v>
-      </c>
-      <c r="C8" s="16">
-        <v>0</v>
-      </c>
-      <c r="D8" s="16">
-        <v>0</v>
-      </c>
-      <c r="E8" s="16">
-        <v>1</v>
-      </c>
-      <c r="F8" s="16">
-        <v>1</v>
-      </c>
-      <c r="G8" s="16">
-        <v>0</v>
-      </c>
-      <c r="H8" s="16">
-        <v>0</v>
-      </c>
-      <c r="I8" s="16">
-        <v>1</v>
-      </c>
-      <c r="K8" s="13">
-        <f>(B8*128+C8*64+D8*32+E8*16+F8*8+G8*4+H8*2+I8*1)</f>
-        <v>153</v>
-      </c>
-    </row>
-    <row r="9" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A9" s="13"/>
-      <c r="B9" s="16">
-        <v>1</v>
-      </c>
-      <c r="C9" s="16">
-        <v>0</v>
-      </c>
-      <c r="D9" s="16">
-        <v>0</v>
-      </c>
-      <c r="E9" s="16">
-        <v>1</v>
-      </c>
-      <c r="F9" s="16">
-        <v>1</v>
-      </c>
-      <c r="G9" s="16">
-        <v>0</v>
-      </c>
-      <c r="H9" s="16">
-        <v>0</v>
-      </c>
-      <c r="I9" s="16">
-        <v>1</v>
-      </c>
-      <c r="K9" s="13">
-        <f>(B9*128+C9*64+D9*32+E9*16+F9*8+G9*4+H9*2+I9*1)</f>
-        <v>153</v>
-      </c>
-    </row>
-    <row r="10" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="A10" s="13"/>
-      <c r="B10" s="16">
-        <v>1</v>
-      </c>
-      <c r="C10" s="16">
-        <v>0</v>
-      </c>
-      <c r="D10" s="16">
-        <v>0</v>
-      </c>
-      <c r="E10" s="16">
-        <v>1</v>
-      </c>
-      <c r="F10" s="16">
-        <v>1</v>
-      </c>
-      <c r="G10" s="16">
-        <v>1</v>
-      </c>
-      <c r="H10" s="16">
-        <v>1</v>
-      </c>
-      <c r="I10" s="16">
-        <v>1</v>
-      </c>
-      <c r="K10" s="13">
-        <f>(B10*128+C10*64+D10*32+E10*16+F10*8+G10*4+H10*2+I10*1)</f>
-        <v>159</v>
-      </c>
-    </row>
-    <row r="11" s="13" customFormat="1" ht="46.799999999999997" customHeight="1">
-      <c r="B11" s="16">
-        <v>1</v>
-      </c>
-      <c r="C11" s="16">
-        <v>1</v>
-      </c>
-      <c r="D11" s="16">
-        <v>1</v>
-      </c>
-      <c r="E11" s="16">
-        <v>1</v>
-      </c>
-      <c r="F11" s="16">
-        <v>1</v>
-      </c>
-      <c r="G11" s="16">
-        <v>1</v>
-      </c>
-      <c r="H11" s="16">
-        <v>1</v>
-      </c>
-      <c r="I11" s="16">
-        <v>1</v>
-      </c>
-      <c r="K11" s="13">
-        <f>(B11*128+C11*64+D11*32+E11*16+F11*8+G11*4+H11*2+I11*1)</f>
+        <v xml:space="preserve">DB 255,129,129,129,129,129,129,255</v>
+      </c>
+      <c r="O4" s="10"/>
+      <c r="P4" s="10"/>
+    </row>
+    <row r="5" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A5" s="10"/>
+      <c r="B5" s="13">
+        <v>1</v>
+      </c>
+      <c r="C5" s="13">
+        <v>0</v>
+      </c>
+      <c r="D5" s="13">
+        <v>0</v>
+      </c>
+      <c r="E5" s="13">
+        <v>0</v>
+      </c>
+      <c r="F5" s="13">
+        <v>0</v>
+      </c>
+      <c r="G5" s="13">
+        <v>0</v>
+      </c>
+      <c r="H5" s="13">
+        <v>0</v>
+      </c>
+      <c r="I5" s="13">
+        <v>1</v>
+      </c>
+      <c r="J5" s="10"/>
+      <c r="K5" s="10">
+        <f t="shared" si="3"/>
+        <v>129</v>
+      </c>
+      <c r="L5" s="10"/>
+      <c r="M5" s="10"/>
+      <c r="N5" s="10"/>
+      <c r="O5" s="10"/>
+      <c r="P5" s="10"/>
+    </row>
+    <row r="6" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A6" s="10"/>
+      <c r="B6" s="13">
+        <v>1</v>
+      </c>
+      <c r="C6" s="13">
+        <v>0</v>
+      </c>
+      <c r="D6" s="13">
+        <v>0</v>
+      </c>
+      <c r="E6" s="13">
+        <v>0</v>
+      </c>
+      <c r="F6" s="13">
+        <v>0</v>
+      </c>
+      <c r="G6" s="13">
+        <v>0</v>
+      </c>
+      <c r="H6" s="13">
+        <v>0</v>
+      </c>
+      <c r="I6" s="13">
+        <v>1</v>
+      </c>
+      <c r="K6" s="10">
+        <f t="shared" si="3"/>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="7" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A7" s="10"/>
+      <c r="B7" s="13">
+        <v>1</v>
+      </c>
+      <c r="C7" s="13">
+        <v>0</v>
+      </c>
+      <c r="D7" s="13">
+        <v>0</v>
+      </c>
+      <c r="E7" s="13">
+        <v>0</v>
+      </c>
+      <c r="F7" s="13">
+        <v>0</v>
+      </c>
+      <c r="G7" s="13">
+        <v>0</v>
+      </c>
+      <c r="H7" s="13">
+        <v>0</v>
+      </c>
+      <c r="I7" s="13">
+        <v>1</v>
+      </c>
+      <c r="K7" s="10">
+        <f t="shared" si="3"/>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="8" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A8" s="10"/>
+      <c r="B8" s="13">
+        <v>1</v>
+      </c>
+      <c r="C8" s="13">
+        <v>0</v>
+      </c>
+      <c r="D8" s="13">
+        <v>0</v>
+      </c>
+      <c r="E8" s="13">
+        <v>0</v>
+      </c>
+      <c r="F8" s="13">
+        <v>0</v>
+      </c>
+      <c r="G8" s="13">
+        <v>0</v>
+      </c>
+      <c r="H8" s="13">
+        <v>0</v>
+      </c>
+      <c r="I8" s="13">
+        <v>1</v>
+      </c>
+      <c r="K8" s="10">
+        <f t="shared" si="3"/>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A9" s="10"/>
+      <c r="B9" s="13">
+        <v>1</v>
+      </c>
+      <c r="C9" s="13">
+        <v>0</v>
+      </c>
+      <c r="D9" s="13">
+        <v>0</v>
+      </c>
+      <c r="E9" s="13">
+        <v>0</v>
+      </c>
+      <c r="F9" s="13">
+        <v>0</v>
+      </c>
+      <c r="G9" s="13">
+        <v>0</v>
+      </c>
+      <c r="H9" s="13">
+        <v>0</v>
+      </c>
+      <c r="I9" s="13">
+        <v>1</v>
+      </c>
+      <c r="K9" s="10">
+        <f t="shared" si="3"/>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="10" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="A10" s="10"/>
+      <c r="B10" s="13">
+        <v>1</v>
+      </c>
+      <c r="C10" s="13">
+        <v>0</v>
+      </c>
+      <c r="D10" s="13">
+        <v>0</v>
+      </c>
+      <c r="E10" s="13">
+        <v>0</v>
+      </c>
+      <c r="F10" s="13">
+        <v>0</v>
+      </c>
+      <c r="G10" s="13">
+        <v>0</v>
+      </c>
+      <c r="H10" s="13">
+        <v>0</v>
+      </c>
+      <c r="I10" s="13">
+        <v>1</v>
+      </c>
+      <c r="K10" s="10">
+        <f t="shared" ref="K10:K11" si="4">(B10*128+C10*64+D10*32+E10*16+F10*8+G10*4+H10*2+I10*1)</f>
+        <v>129</v>
+      </c>
+    </row>
+    <row r="11" s="10" customFormat="1" ht="46.799999999999997" customHeight="1">
+      <c r="B11" s="13">
+        <v>1</v>
+      </c>
+      <c r="C11" s="13">
+        <v>1</v>
+      </c>
+      <c r="D11" s="13">
+        <v>1</v>
+      </c>
+      <c r="E11" s="13">
+        <v>1</v>
+      </c>
+      <c r="F11" s="13">
+        <v>1</v>
+      </c>
+      <c r="G11" s="13">
+        <v>1</v>
+      </c>
+      <c r="H11" s="13">
+        <v>1</v>
+      </c>
+      <c r="I11" s="13">
+        <v>1</v>
+      </c>
+      <c r="K11" s="10">
+        <f t="shared" si="4"/>
         <v>255</v>
       </c>
     </row>
@@ -1264,7 +1253,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{362258E5-24AA-412C-981D-85FB3F253538}">
+          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{4FD5D10D-614B-4665-9378-CEB1AAAC5112}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1281,7 +1270,7 @@
           <xm:sqref>B4:I4</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{7094EB36-22B3-4342-B941-E098D462C267}">
+          <x14:cfRule type="cellIs" priority="2" operator="greaterThan" id="{6914A121-0489-4C81-9D9B-9969C083B379}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1298,7 +1287,7 @@
           <xm:sqref>B5:I5</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{AB507B41-E923-420B-9BAF-D12B18A52279}">
+          <x14:cfRule type="cellIs" priority="3" operator="greaterThan" id="{5B95A5B9-22CB-45E6-91A0-EC2CD69570DB}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1315,7 +1304,7 @@
           <xm:sqref>B6:I6</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{F834099C-2313-4F86-B19D-52A920703A52}">
+          <x14:cfRule type="cellIs" priority="4" operator="greaterThan" id="{B19519E8-DEB7-4807-85CD-B0290BA3BBDF}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1332,7 +1321,7 @@
           <xm:sqref>B7:I7</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{3DB18D29-751A-4465-9DF6-F79154B6D331}">
+          <x14:cfRule type="cellIs" priority="5" operator="greaterThan" id="{618C2AC7-10E4-4296-8390-1DFAB2D0E7A9}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1349,7 +1338,7 @@
           <xm:sqref>B8:I8</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{8FD071FD-D041-4CA8-A91D-C49B8ADDFEA7}">
+          <x14:cfRule type="cellIs" priority="6" operator="greaterThan" id="{976F1449-0366-42F2-9A30-804C6633CCF2}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1366,7 +1355,7 @@
           <xm:sqref>B9:I9</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{568DA1F3-ECA5-425D-8CD1-A58BA40D5838}">
+          <x14:cfRule type="cellIs" priority="7" operator="greaterThan" id="{6DBB72A8-9100-480E-95BD-F2C89ACB99A7}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>
@@ -1383,7 +1372,7 @@
           <xm:sqref>B10:I10</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="cellIs" priority="1" operator="greaterThan" id="{7AD793B5-D3F7-413C-92DA-2E0CD79B0DD7}">
+          <x14:cfRule type="cellIs" priority="8" operator="greaterThan" id="{3C70C287-547F-4068-A068-EA654E3DE89D}">
             <xm:f>0</xm:f>
             <x14:dxf>
               <font>

</xml_diff>